<commit_message>
modified rounded numbers in table
</commit_message>
<xml_diff>
--- a/out/Summary_table.xlsx
+++ b/out/Summary_table.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$I$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -50,87 +53,88 @@
     <t>OAE</t>
   </si>
   <si>
-    <t>Alkalinity 
-[μmol kg-1]</t>
-  </si>
-  <si>
-    <t>(2198.155, 2210.332)</t>
-  </si>
-  <si>
-    <t>(2314.785, 
-2327.401)</t>
-  </si>
-  <si>
-    <t>(2167.332, 
-2184.407)</t>
-  </si>
-  <si>
-    <t>(2297.88, 
-2314.238)</t>
-  </si>
-  <si>
-    <t>(2184.39, 
-2203.275)</t>
-  </si>
-  <si>
-    <t>(2563.496, 
-2671.551)</t>
-  </si>
-  <si>
-    <t>(2137.895, 
-2161.921)</t>
-  </si>
-  <si>
-    <t>(2546.925, 
-2684.538)</t>
-  </si>
-  <si>
-    <t>Surface ocean pCO2 
-[μatm]</t>
-  </si>
-  <si>
-    <t>(403.918, 
-433.014)</t>
-  </si>
-  <si>
-    <t>(356.824, 
-373.648)</t>
-  </si>
-  <si>
-    <t>(744.658, 
-807.266)</t>
-  </si>
-  <si>
-    <t>(674.444, 
-719.006)</t>
-  </si>
-  <si>
-    <t>(390.772, 
-452.232)</t>
-  </si>
-  <si>
-    <t>(187.505, 
-237.542)</t>
-  </si>
-  <si>
-    <t>(730.434, 
-835.971)</t>
-  </si>
-  <si>
-    <t>(344.042, 
-460.916)</t>
+    <t>Alkalinity
+ [μmol kg-1]</t>
+  </si>
+  <si>
+    <t>(2198, 
+2210)</t>
+  </si>
+  <si>
+    <t>(2315, 
+2327)</t>
+  </si>
+  <si>
+    <t>(2167, 
+2184)</t>
+  </si>
+  <si>
+    <t>(2298, 
+2314)</t>
+  </si>
+  <si>
+    <t>(2184, 
+2203)</t>
+  </si>
+  <si>
+    <t>(2563, 
+2672)</t>
+  </si>
+  <si>
+    <t>(2138, 
+2162)</t>
+  </si>
+  <si>
+    <t>(2547,
+ 2685)</t>
+  </si>
+  <si>
+    <t>Surface ocean pCO2
+ [μatm]</t>
+  </si>
+  <si>
+    <t>(404, 
+433)</t>
+  </si>
+  <si>
+    <t>(357, 
+374)</t>
+  </si>
+  <si>
+    <t>(745, 
+807)</t>
+  </si>
+  <si>
+    <t>(674, 
+719)</t>
+  </si>
+  <si>
+    <t>(391, 
+452)</t>
+  </si>
+  <si>
+    <t>(188, 
+238)</t>
+  </si>
+  <si>
+    <t>(730, 
+836)</t>
+  </si>
+  <si>
+    <t>(344, 
+461)</t>
   </si>
   <si>
     <t>Air-sea CO2 flux
- [kg-1 m-2 y-1]</t>
+ [kg m-2 y-1]</t>
   </si>
   <si>
     <t>(-0.102, 
 0.009)</t>
   </si>
   <si>
-    <t>(-0.235, 
--0.067)</t>
+    <t>(-0.235,
+ -0.067)</t>
   </si>
   <si>
     <t>(-0.142, 
@@ -157,40 +161,40 @@
 -0.318)</t>
   </si>
   <si>
-    <t>Mixed layer depth 
-[m]</t>
-  </si>
-  <si>
-    <t>(15.259, 
-135.275)</t>
-  </si>
-  <si>
-    <t>(15.302, 
-141.488)</t>
-  </si>
-  <si>
-    <t>(14.25, 
-107.422)</t>
-  </si>
-  <si>
-    <t>(14.054, 
-105.835)</t>
-  </si>
-  <si>
-    <t>(14.866, 
-76.167)</t>
-  </si>
-  <si>
-    <t>(15.086, 
-75.48)</t>
-  </si>
-  <si>
-    <t>(13.936, 
-67.561)</t>
-  </si>
-  <si>
-    <t>(14.097, 
-66.18)</t>
+    <t>Mixed layer depth
+ [m]</t>
+  </si>
+  <si>
+    <t>(15, 
+135)</t>
+  </si>
+  <si>
+    <t>(15, 
+141)</t>
+  </si>
+  <si>
+    <t>(14, 
+107)</t>
+  </si>
+  <si>
+    <t>(14, 
+106)</t>
+  </si>
+  <si>
+    <t>(15, 
+76)</t>
+  </si>
+  <si>
+    <t>(15,
+ 75)</t>
+  </si>
+  <si>
+    <t>(14, 
+68)</t>
+  </si>
+  <si>
+    <t>(14, 
+66)</t>
   </si>
 </sst>
 </file>
@@ -203,7 +207,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,14 +216,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Georgia Regular"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
+      <sz val="12"/>
+      <name val="Georgia Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Georgia Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8"/>
       <name val="Georgia Regular"/>
       <charset val="134"/>
     </font>
@@ -569,7 +584,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -581,6 +596,17 @@
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -615,51 +641,6 @@
         <color auto="1"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
         <color auto="1"/>
       </top>
       <bottom style="thin">
@@ -677,24 +658,185 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="medium">
         <color auto="1"/>
       </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -702,19 +844,12 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -821,28 +956,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -851,172 +977,211 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1364,22 +1529,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultColWidth="10.1160714285714" defaultRowHeight="14.4" outlineLevelRow="7"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultColWidth="8.92857142857143" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="1" width="19.1071428571429" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.92857142857143" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9.10714285714286" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.75" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.92857142857143" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.46428571428571" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.10714285714286" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.66964285714286" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.1160714285714" style="1" customWidth="1"/>
+    <col min="1" max="1" width="23.3928571428571" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.2142857142857" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.57142857142857" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.2142857142857" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.48214285714286" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.2142857142857" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.57142857142857" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.2142857142857" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.75" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.92857142857143" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:9">
+    <row r="1" ht="17.6" spans="1:10">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1389,180 +1557,177 @@
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="5"/>
+      <c r="I1" s="6"/>
     </row>
-    <row r="2" ht="15" spans="1:9">
-      <c r="A2" s="6" t="s">
+    <row r="2" ht="17.6" spans="1:10">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="7" t="s">
+      <c r="E2" s="9"/>
+      <c r="F2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="7" t="s">
+      <c r="G2" s="9"/>
+      <c r="H2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="9"/>
+      <c r="I2" s="11"/>
     </row>
-    <row r="3" ht="15" spans="1:9">
-      <c r="A3" s="6" t="s">
+    <row r="3" ht="18.35" spans="1:10">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="11"/>
-      <c r="I4" s="12"/>
+    <row r="4" ht="36" spans="1:10">
+      <c r="A4" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="5" ht="29" spans="1:9">
-      <c r="A5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>15</v>
-      </c>
+    <row r="5" ht="36" spans="1:10">
+      <c r="A5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="23"/>
     </row>
-    <row r="6" ht="29" spans="1:9">
-      <c r="A6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>24</v>
+    <row r="6" ht="36" spans="1:10">
+      <c r="A6" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="22" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="7" ht="29" spans="1:9">
-      <c r="A7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" ht="29.75" spans="1:9">
-      <c r="A8" s="15" t="s">
+    <row r="7" ht="36.75" spans="1:10">
+      <c r="A7" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B7" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C7" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D7" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E7" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F7" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G7" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H7" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="I7" s="27" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1576,7 +1741,7 @@
     <mergeCell ref="H2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="256" orientation="landscape"/>
+  <pageSetup paperSize="11" scale="88" orientation="landscape"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>